<commit_message>
feat: export autonome de la feuille touches et melees
</commit_message>
<xml_diff>
--- a/Matchs/26-27_A2_Panjas-AC_Premiere_EXT - Touches et melees.xlsx
+++ b/Matchs/26-27_A2_Panjas-AC_Premiere_EXT - Touches et melees.xlsx
@@ -8,85 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bastiendallago/Library/Mobile Documents/com~apple~CloudDocs/Documents/DD/1- PERSO/12- AUTRES/1- RUGBY/2026-2027 MXV/STAT_VEO/Matchs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{695BBE21-E0BF-2E42-93CD-FA0AA553F306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F054F08-6201-7243-BDB6-6A2F767D18F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" xr2:uid="{86F2EA48-CD00-C548-B51B-46220ACFFC4F}"/>
+    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" xr2:uid="{049E49DC-62EB-A441-A8EA-2B9592944B0A}"/>
   </bookViews>
   <sheets>
     <sheet name="Touches Melees" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
-  <definedNames>
-    <definedName name="ACT_ATT_NULLE">[1]Paramètres!$R$53</definedName>
-    <definedName name="ACT_AVANCEE">[1]Paramètres!$R$54</definedName>
-    <definedName name="ACT_FRANCHISSEMENT">[1]Paramètres!$R$42</definedName>
-    <definedName name="ACT_ME_ADV_G">[1]Paramètres!$R$40</definedName>
-    <definedName name="ACT_ME_ADV_P">[1]Paramètres!$R$41</definedName>
-    <definedName name="ACT_ME_NS_G">[1]Paramètres!$R$38</definedName>
-    <definedName name="ACT_ME_NS_P">[1]Paramètres!$R$39</definedName>
-    <definedName name="ACT_PEN_CONTRE_ADV">[1]Paramètres!$R$13</definedName>
-    <definedName name="ACT_PEN_CONTRE_NOUS">[1]Paramètres!$R$14</definedName>
-    <definedName name="ACT_PEN_HORS_JEU">[1]Paramètres!$R$33</definedName>
-    <definedName name="ACT_PEN_MAUL">[1]Paramètres!$R$31</definedName>
-    <definedName name="ACT_PEN_PL_A_2">[1]Paramètres!$R$34</definedName>
-    <definedName name="ACT_PEN_PL_HAUT">[1]Paramètres!$R$35</definedName>
-    <definedName name="ACT_PEN_RUCK">[1]Paramètres!$R$32</definedName>
-    <definedName name="ACT_PEN_UNKNOWN">[1]Paramètres!$R$36</definedName>
-    <definedName name="ACT_PL_A2">[1]Paramètres!$R$5</definedName>
-    <definedName name="ACT_PL_HAUT">[1]Paramètres!$R$6</definedName>
-    <definedName name="ACT_PL_NORMAL">[1]Paramètres!$R$3</definedName>
-    <definedName name="ACT_PL_OFF">[1]Paramètres!$R$2</definedName>
-    <definedName name="ACT_PL_RATE">[1]Paramètres!$R$4</definedName>
-    <definedName name="ACT_PTS_DROP">[1]Paramètres!$R$19</definedName>
-    <definedName name="ACT_PTS_ESSAI">[1]Paramètres!$R$15</definedName>
-    <definedName name="ACT_PTS_ESSAI_PEN">[1]Paramètres!$R$16</definedName>
-    <definedName name="ACT_PTS_PENALITE">[1]Paramètres!$R$18</definedName>
-    <definedName name="ACT_PTS_TRANSFO">[1]Paramètres!$R$17</definedName>
-    <definedName name="ACT_TO_ADV_PAS_DROIT">[1]Paramètres!$R$12</definedName>
-    <definedName name="ACT_TO_ADV_PERDUE">[1]Paramètres!$R$11</definedName>
-    <definedName name="ACT_TO_ADV_VOLEE">[1]Paramètres!$R$10</definedName>
-    <definedName name="ACT_TO_NS_G">[1]Paramètres!$R$7</definedName>
-    <definedName name="ACT_TO_NS_P">[1]Paramètres!$R$8</definedName>
-    <definedName name="ACT_TO_NS_PAS_DROIT">[1]Paramètres!$R$9</definedName>
-    <definedName name="AVANT_OU_ARRIERE">[1]!LstLignePoste[AVANT_OU_ARRIERE]</definedName>
-    <definedName name="BTNS_JOUEURS">'[1]Saisie vidéo'!$D$14,'[1]Saisie vidéo'!$F$14,'[1]Saisie vidéo'!$H$14,'[1]Saisie vidéo'!$J$14,'[1]Saisie vidéo'!$L$14,'[1]Saisie vidéo'!$N$14,'[1]Saisie vidéo'!$N$16,'[1]Saisie vidéo'!$L$16,'[1]Saisie vidéo'!$J$16,'[1]Saisie vidéo'!$H$16,'[1]Saisie vidéo'!$F$16</definedName>
-    <definedName name="EQUIPE_NIV">[1]!LstEquipesClub[EQUIPE_NIV]</definedName>
-    <definedName name="EQUIPES_POULE">[1]!LstEquipesPoule[EQUIPES_A_AFFRONTER]</definedName>
-    <definedName name="LIEU_MATCH">[1]!LstLieuxMatch[LIEU_MATCH]</definedName>
-    <definedName name="LISTE_ACTIONS_JOURNAL">[1]!TblActionsJournal[Libellé]</definedName>
-    <definedName name="LISTE_EQUIPES_JOURNAL">[1]!TblEquipesJournal[LISTE_EQUIPES_JOURNAL]</definedName>
-    <definedName name="LISTE_GROUPES_FAUTIFS">[1]!LstLignePoste[AVANT_OU_ARRIERE]</definedName>
-    <definedName name="LISTE_JOUEURS">[1]!LstEffectif[prenom NOM]</definedName>
-    <definedName name="LISTE_JOUEURS_JOURNAL">[1]!LstJoueursJournal[LISTE_JOUEURS_JOURNAL]</definedName>
-    <definedName name="LISTE_LECTEURS_VIDEO">[1]!TblLecteurVideo[LISTE_LECTEUR_VIDEO]</definedName>
-    <definedName name="LISTE_MOTIFS_PENALITE">[1]Paramètres!$R$31:$R$36</definedName>
-    <definedName name="LISTE_MT_JOURNAL">[1]Paramètres!$I$6:$I$7</definedName>
-    <definedName name="LST_JOUEURS">[1]!LstEffectif[NOM Prénom]</definedName>
-    <definedName name="LST_TM_ALIGNEMENT">'Touches Melees'!$AC$2:$AC$7</definedName>
-    <definedName name="LST_TM_BALLON">'Touches Melees'!$AA$2:$AA$3</definedName>
-    <definedName name="LST_TM_BALLON_LONG">'Touches Melees'!$AF$2:$AF$3</definedName>
-    <definedName name="LST_TM_ISSUE_MELEE">'Touches Melees'!$Y$2:$Y$3</definedName>
-    <definedName name="LST_TM_ISSUE_TOUCHE">'Touches Melees'!$X$2:$X$4</definedName>
-    <definedName name="LST_TM_LANCE_POUR">'Touches Melees'!$W$2:$W$3</definedName>
-    <definedName name="LST_TM_UTILISATION">'Touches Melees'!$AE$2:$AE$4</definedName>
-    <definedName name="LST_TM_ZONE_LARGEUR">'Touches Melees'!$AD$2:$AD$4</definedName>
-    <definedName name="LST_TM_ZONE_LONGUEUR">'Touches Melees'!$AB$2:$AB$12</definedName>
-    <definedName name="LST_TM_ZONE_SAUT">'Touches Melees'!$Z$2:$Z$6</definedName>
-    <definedName name="LSTResultat">[1]!Tableau14[[#All],[RESULTAT]]</definedName>
-    <definedName name="MATCH_ADV">[1]Compo!$C$12</definedName>
-    <definedName name="MATCH_CAT">[1]Compo!$C$22</definedName>
-    <definedName name="MATCH_JOURNEE">[1]Compo!$C$18</definedName>
-    <definedName name="MATCH_LIEU">[1]Compo!$C$14</definedName>
-    <definedName name="MATCH_NOUS">[1]Compo!$C$10</definedName>
-    <definedName name="MATCH_PHASE">[1]Compo!$C$16</definedName>
-    <definedName name="OUI_NON">[1]!Tableau15[OUI_NON]</definedName>
-    <definedName name="PHASE">[1]!LstPhases[PHASE]</definedName>
-    <definedName name="RESULTAT">[1]!Tableau14[RESULTAT]</definedName>
-    <definedName name="TM_RECAP_MELEES">'Touches Melees'!$L$19</definedName>
-    <definedName name="TM_RECAP_TOUCHES">'Touches Melees'!$A$25</definedName>
-  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -111,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="62">
   <si>
     <t>TOUCHES</t>
   </si>
@@ -119,36 +47,6 @@
     <t>MELEES</t>
   </si>
   <si>
-    <t>LST_TM_LANCE_POUR</t>
-  </si>
-  <si>
-    <t>LST_TM_ISSUE_TOUCHE</t>
-  </si>
-  <si>
-    <t>LST_TM_ISSUE_MELEE</t>
-  </si>
-  <si>
-    <t>LST_TM_ZONE_SAUT</t>
-  </si>
-  <si>
-    <t>LST_TM_BALLON</t>
-  </si>
-  <si>
-    <t>LST_TM_ZONE_LONGUEUR</t>
-  </si>
-  <si>
-    <t>LST_TM_ALIGNEMENT</t>
-  </si>
-  <si>
-    <t>LST_TM_ZONE_LARGEUR</t>
-  </si>
-  <si>
-    <t>LST_TM_UTILISATION</t>
-  </si>
-  <si>
-    <t>LST_TM_BALLON_LONG</t>
-  </si>
-  <si>
     <t>Temps video</t>
   </si>
   <si>
@@ -215,12 +113,6 @@
     <t>Gauche</t>
   </si>
   <si>
-    <t>Avants</t>
-  </si>
-  <si>
-    <t>Chaud</t>
-  </si>
-  <si>
     <t>MT1</t>
   </si>
   <si>
@@ -263,12 +155,6 @@
     <t>N 15m</t>
   </si>
   <si>
-    <t>Trois-quart</t>
-  </si>
-  <si>
-    <t>Froid</t>
-  </si>
-  <si>
     <t>BARATGIN Julian</t>
   </si>
   <si>
@@ -290,9 +176,6 @@
     <t>N 22m</t>
   </si>
   <si>
-    <t>Pied</t>
-  </si>
-  <si>
     <t>E 40m</t>
   </si>
   <si>
@@ -305,9 +188,6 @@
     <t>Z3</t>
   </si>
   <si>
-    <t>E 22m</t>
-  </si>
-  <si>
     <t>MT2</t>
   </si>
   <si>
@@ -317,7 +197,10 @@
     <t>Sauteur lobbé</t>
   </si>
   <si>
-    <t>E en-but</t>
+    <t>Pas de zone – personne à saut</t>
+  </si>
+  <si>
+    <t>ou Z1,5?</t>
   </si>
   <si>
     <t>2 relayeurs</t>
@@ -353,10 +236,11 @@
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -432,14 +316,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -468,7 +351,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -607,319 +493,39 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Listes"/>
-      <sheetName val="Compo"/>
-      <sheetName val="Saisie vidéo"/>
-      <sheetName val="Journal actions"/>
-      <sheetName val="Stats match"/>
-      <sheetName val="Touches Melees"/>
-      <sheetName val="Paramètres"/>
-      <sheetName val="Popup"/>
-      <sheetName val="Popup touche"/>
-      <sheetName val="Popup melee"/>
-      <sheetName val="Popup penalite"/>
-      <sheetName val="Popup remplacement"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="10">
-          <cell r="C10" t="str">
-            <v>MXV</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="C12" t="str">
-            <v>Panjas AC</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="C14" t="str">
-            <v>Extérieur</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="C16" t="str">
-            <v>Aller</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="C18">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="C22" t="str">
-            <v>Première</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2">
-        <row r="14">
-          <cell r="D14" t="str">
-            <v>1
-ABADIE</v>
-          </cell>
-          <cell r="F14" t="str">
-            <v>2
-RICHIARDONNE</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>3
-BAUP</v>
-          </cell>
-          <cell r="J14" t="str">
-            <v>4
-DUTREY</v>
-          </cell>
-          <cell r="L14" t="str">
-            <v>5
-ABADIE</v>
-          </cell>
-          <cell r="N14" t="str">
-            <v>6
-MULLIER</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="F16" t="str">
-            <v>8
-BARATGIN</v>
-          </cell>
-          <cell r="H16" t="str">
-            <v>9
-MOUDENS</v>
-          </cell>
-          <cell r="J16" t="str">
-            <v>10
-COURREGES</v>
-          </cell>
-          <cell r="L16" t="str">
-            <v>11
-BOURREC</v>
-          </cell>
-          <cell r="N16" t="str">
-            <v>12
-LAUDET</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6">
-        <row r="2">
-          <cell r="R2" t="str">
-            <v>Plaquage offensif</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="R3" t="str">
-            <v>Plaquage normal</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="R4" t="str">
-            <v>Plaquage raté</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="R5" t="str">
-            <v>Plaquage à 2</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="I6" t="str">
-            <v>MT1</v>
-          </cell>
-          <cell r="R6" t="str">
-            <v>Plaquage haut</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="I7" t="str">
-            <v>MT2</v>
-          </cell>
-          <cell r="R7" t="str">
-            <v>Touche à nous conservée</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="R8" t="str">
-            <v>Touche à nous perdue</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="R9" t="str">
-            <v>Touche à nous pas droite</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="R10" t="str">
-            <v>Touche à eux volée</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="R11" t="str">
-            <v>Touche à eux perdue</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="R12" t="str">
-            <v>Touche à eux pas droite</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="R13" t="str">
-            <v>Pénalité contre adversaire</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="R14" t="str">
-            <v>Pénalité contre nous</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="R15" t="str">
-            <v>Essai</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="R16" t="str">
-            <v>Essai de pénalité</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="R17" t="str">
-            <v>Transformation</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="R18" t="str">
-            <v>Pénalité</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="R19" t="str">
-            <v>Drop</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="R31" t="str">
-            <v>Maul</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="R32" t="str">
-            <v>Ruck</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="R33" t="str">
-            <v>Hors-jeu</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="R34" t="str">
-            <v>Plaquage à 2</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="R35" t="str">
-            <v>Plaquage haut</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="R36" t="str">
-            <v>?</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="R38" t="str">
-            <v>Mêlée à nous gagnée</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="R39" t="str">
-            <v>Mêlée à nous perdue</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="R40" t="str">
-            <v>Mêlée à eux volée</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="R41" t="str">
-            <v>Mêlée à eux perdue</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="R42" t="str">
-            <v>Franchissement</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="R53" t="str">
-            <v>Recul ou sans progression</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="R54" t="str">
-            <v>Avancée au contact</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C634A84-E7C3-A34D-8E47-CC8D50C31335}" name="DetailTouches" displayName="DetailTouches" ref="A2:J24" totalsRowShown="0">
-  <autoFilter ref="A2:J24" xr:uid="{1BC259CC-2467-644D-900B-02D4F95FCC56}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{174EE8B9-1050-E946-84E3-DA3BBB6009F5}" name="DetailTouches" displayName="DetailTouches" ref="A2:J24" totalsRowShown="0">
+  <autoFilter ref="A2:J24" xr:uid="{174EE8B9-1050-E946-84E3-DA3BBB6009F5}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{324D563E-2DCE-1643-9065-D44D495DDA7D}" name="Temps video" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{647D539D-7013-3A43-8CF2-FFBCB547217E}" name="Mi-temps"/>
-    <tableColumn id="3" xr3:uid="{72096FC7-CA5C-C846-B0AD-A7A653B75FA7}" name="Lance pour"/>
-    <tableColumn id="4" xr3:uid="{3C37FD53-1865-7840-BCFF-5190D7FAE143}" name="Issue"/>
-    <tableColumn id="5" xr3:uid="{BB98D75A-3ADB-5A47-B7A3-552B9BC232D4}" name="Sauteur"/>
-    <tableColumn id="6" xr3:uid="{DF2CE184-05D2-604E-84A8-2DF1431362F9}" name="Zone saut"/>
-    <tableColumn id="7" xr3:uid="{8C2BAA64-0E60-3A4D-93BC-43A7E6724F26}" name="Ballon"/>
-    <tableColumn id="8" xr3:uid="{D402ED8C-61B4-C049-8AE2-6C62B02EBA8F}" name="Zone terrain"/>
-    <tableColumn id="9" xr3:uid="{3151BB58-9002-3844-9ED6-6E411D0151CC}" name="Alignement"/>
-    <tableColumn id="10" xr3:uid="{6F3B9780-0E5F-4744-920A-6666E492231B}" name="Observations"/>
+    <tableColumn id="1" xr3:uid="{FEBA0587-E449-8044-89AF-1C46216C41F7}" name="Temps video" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{0458A7B7-7123-BB4B-9699-4DE89AFC8F11}" name="Mi-temps"/>
+    <tableColumn id="3" xr3:uid="{31BA59A2-BBA2-8247-BD5E-309E080F117D}" name="Lance pour"/>
+    <tableColumn id="4" xr3:uid="{BEAFE920-D055-C843-A579-8D6C85A86EA2}" name="Issue"/>
+    <tableColumn id="5" xr3:uid="{0FD9EC8B-3D38-F346-AA55-A4B098491D76}" name="Sauteur"/>
+    <tableColumn id="6" xr3:uid="{A47B2AD8-C0A5-BE4E-B60D-459E56AB64C3}" name="Zone saut"/>
+    <tableColumn id="7" xr3:uid="{918A80F2-C063-3748-A2F5-A71B558FFF2F}" name="Ballon"/>
+    <tableColumn id="8" xr3:uid="{36D66329-4C7E-7242-AE16-6039504881F7}" name="Zone terrain"/>
+    <tableColumn id="9" xr3:uid="{A794EF41-A9A9-B845-A13A-3C906BFDFAD3}" name="Alignement"/>
+    <tableColumn id="10" xr3:uid="{CDC5671A-DD8C-A648-B14C-7E44091A13DF}" name="Observations"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7E9E174D-7278-4743-AECF-EEA4E668FDA8}" name="DetailMelees" displayName="DetailMelees" ref="L2:U17" totalsRowShown="0">
-  <autoFilter ref="L2:U17" xr:uid="{A1FE138B-7A57-FD4E-B0BC-4BF4203BE379}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6AF0E287-0BE8-E444-B349-8449D74EED98}" name="DetailMelees" displayName="DetailMelees" ref="L2:U17" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="L2:U17" xr:uid="{6AF0E287-0BE8-E444-B349-8449D74EED98}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{1A5FA3EA-049E-F644-9A24-5BDE14023051}" name="Temps video" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{46245036-4524-964D-A0EE-EAA9F538CF0F}" name="Mi-temps"/>
-    <tableColumn id="3" xr3:uid="{25EBF3C1-F0C3-5042-AD94-2269E431A67F}" name="Introduction pour"/>
-    <tableColumn id="4" xr3:uid="{83016B1D-2DBA-FF48-B440-2C5A81D15686}" name="Issue"/>
-    <tableColumn id="5" xr3:uid="{E239AF70-A65C-B848-A00B-A44FCAE3D417}" name="Zone longueur"/>
-    <tableColumn id="6" xr3:uid="{E2AF864C-EF84-D14C-9D27-D2F007128899}" name="Zone largeur"/>
-    <tableColumn id="7" xr3:uid="{E06B4277-A4CC-B34A-BFFF-1EE5CC024185}" name="Jeu avant" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{6C079AC1-FD2A-2548-8771-A6528C22B9F9}" name="Jeu 3/4" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{BDCED364-EC12-254A-B1FB-B6918ADEBFA7}" name="Jeu pied" dataDxfId="0"/>
-    <tableColumn id="10" xr3:uid="{A66EB1AB-59B3-9D40-875C-16CAADB5DF21}" name="Observations"/>
+    <tableColumn id="1" xr3:uid="{C8259CE3-6AC4-9D46-8B9E-381861CFECEE}" name="Temps video" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{52ACCED4-48BE-4344-B2FD-F76667E51C12}" name="Mi-temps"/>
+    <tableColumn id="3" xr3:uid="{D779FCDC-BEE8-B542-BA13-7122C7510AB5}" name="Introduction pour"/>
+    <tableColumn id="4" xr3:uid="{8B6CC3C5-7E96-2340-B5B6-8A7B0580F906}" name="Issue"/>
+    <tableColumn id="5" xr3:uid="{E1836020-DD7C-4A42-A93F-AF8A1210D599}" name="Zone longueur"/>
+    <tableColumn id="6" xr3:uid="{037C994D-185B-E24F-B3E7-C9033B950F22}" name="Zone largeur"/>
+    <tableColumn id="7" xr3:uid="{F5D570DD-1991-F94A-93EE-31693739C13D}" name="Jeu avant" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{5FD9B417-3912-FA44-ACDD-DC51E85FF1E0}" name="Jeu 3/4" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{6D49C3D8-4582-E64C-B104-418E26876358}" name="Jeu pied" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{AEC07899-12A6-8344-97AD-583CD0311EF7}" name="Observations"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1241,329 +847,227 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4470BB4C-0B8D-D84A-ADCD-6ACFDAA611E0}">
-  <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:AF27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A26FCC8-44A6-1645-BFA4-F760BA6B4F32}">
+  <dimension ref="A1:U28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
     <col min="10" max="10" width="31" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3.83203125" customWidth="1"/>
     <col min="12" max="12" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="20" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="17.5" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="15" customWidth="1"/>
+    <col min="17" max="17" width="13.6640625" customWidth="1"/>
+    <col min="18" max="20" width="12.83203125" customWidth="1"/>
     <col min="21" max="21" width="30.83203125" customWidth="1"/>
-    <col min="22" max="22" width="0" hidden="1" customWidth="1"/>
-    <col min="23" max="32" width="10.83203125" hidden="1" customWidth="1"/>
+    <col min="22" max="52" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="W1" t="s">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="X1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="G2" t="s">
         <v>8</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="H2" t="s">
         <v>9</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="I2" t="s">
         <v>10</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="J2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.15">
-      <c r="A2" t="s">
+      <c r="L2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="O2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="Q2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="R2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="S2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
+      <c r="T2" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>24</v>
-      </c>
-      <c r="R2" t="s">
-        <v>25</v>
-      </c>
-      <c r="S2" t="s">
-        <v>26</v>
-      </c>
-      <c r="T2" t="s">
-        <v>27</v>
-      </c>
       <c r="U2" t="s">
-        <v>21</v>
-      </c>
-      <c r="W2" t="s">
-        <v>28</v>
-      </c>
-      <c r="X2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AC2">
-        <v>2</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.15">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>6.2463804166666666E-3</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
         <v>28</v>
       </c>
-      <c r="D3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H3" t="s">
-        <v>40</v>
-      </c>
       <c r="I3" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="J3" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L3" s="2">
         <v>1.5196666087962962E-3</v>
       </c>
       <c r="M3" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N3" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O3" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P3" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="Q3" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
-      <c r="W3" t="s">
-        <v>46</v>
-      </c>
-      <c r="X3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>47</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>49</v>
-      </c>
-      <c r="AC3">
-        <v>3</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>44</v>
-      </c>
-      <c r="AE3" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.15">
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>7.570339155092593E-3</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
         <v>29</v>
-      </c>
-      <c r="E4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" t="s">
-        <v>41</v>
       </c>
       <c r="L4" s="2">
         <v>3.5945389351851854E-3</v>
       </c>
       <c r="M4" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N4" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O4" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P4" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="Q4" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="T4" s="3"/>
       <c r="U4" t="s">
-        <v>55</v>
-      </c>
-      <c r="X4" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>57</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>58</v>
-      </c>
-      <c r="AC4">
-        <v>4</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>54</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.15">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>8.774028159722223E-3</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>42</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="I5">
         <v>6</v>
@@ -1572,117 +1076,99 @@
         <v>9.1330586689814808E-3</v>
       </c>
       <c r="M5" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N5" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O5" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P5" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="Q5" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="T5" s="3"/>
-      <c r="Z5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.15">
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>1.2905092592592593E-2</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="J6" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L6" s="2">
         <v>1.9498069814814813E-2</v>
       </c>
       <c r="M6" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N6" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="P6" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="Q6" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="T6" s="3"/>
-      <c r="Z6" t="s">
-        <v>63</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>62</v>
-      </c>
-      <c r="AC6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.15">
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>1.3936346412037037E-2</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="F7" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="H7" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="I7">
         <v>6</v>
@@ -1691,47 +1177,44 @@
         <v>2.2532352314814815E-2</v>
       </c>
       <c r="M7" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N7" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O7" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P7" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="Q7" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="T7" s="3"/>
-      <c r="AB7" t="s">
-        <v>43</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.15">
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>1.4201970405092591E-2</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" t="s">
         <v>37</v>
-      </c>
-      <c r="H8" t="s">
-        <v>49</v>
       </c>
       <c r="I8">
         <v>6</v>
@@ -1740,50 +1223,47 @@
         <v>2.3040061608796295E-2</v>
       </c>
       <c r="M8" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N8" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="O8" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="P8" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="Q8" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.15">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>1.6917279039351852E-2</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="H9" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="I9">
         <v>5</v>
@@ -1792,47 +1272,44 @@
         <v>2.3721624803240738E-2</v>
       </c>
       <c r="M9" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N9" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="O9" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="P9" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q9" t="s">
         <v>40</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>54</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.15">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>1.7881212893518517E-2</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="I10">
         <v>4</v>
@@ -1841,47 +1318,44 @@
         <v>2.5400932534722222E-2</v>
       </c>
       <c r="M10" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N10" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O10" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P10" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="Q10" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.15">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>1.8519158668981482E-2</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H11" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="I11">
         <v>5</v>
@@ -1890,102 +1364,99 @@
         <v>3.3542458194444444E-2</v>
       </c>
       <c r="M11" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="N11" t="s">
+        <v>18</v>
+      </c>
+      <c r="O11" t="s">
+        <v>19</v>
+      </c>
+      <c r="P11" t="s">
         <v>28</v>
       </c>
-      <c r="O11" t="s">
-        <v>29</v>
-      </c>
-      <c r="P11" t="s">
-        <v>40</v>
-      </c>
       <c r="Q11" t="s">
+        <v>23</v>
+      </c>
+      <c r="R11" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="R11" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="U11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.15">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>1.9040562418981482E-2</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>19</v>
+      </c>
+      <c r="F12" t="s">
+        <v>27</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I12">
         <v>4</v>
       </c>
       <c r="J12" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="L12" s="2">
         <v>3.5299767303240741E-2</v>
       </c>
       <c r="M12" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="N12" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="O12" t="s">
+        <v>25</v>
+      </c>
+      <c r="P12" t="s">
         <v>37</v>
       </c>
-      <c r="P12" t="s">
-        <v>49</v>
-      </c>
       <c r="Q12" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="R12" s="3"/>
       <c r="S12" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="T12" s="3"/>
-      <c r="AB12" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.15">
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>2.1946519351851854E-2</v>
       </c>
       <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" t="s">
         <v>36</v>
       </c>
-      <c r="C13" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" t="s">
-        <v>48</v>
-      </c>
       <c r="H13" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="I13">
         <v>5</v>
@@ -1994,47 +1465,47 @@
         <v>3.5947130347222224E-2</v>
       </c>
       <c r="M13" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="N13" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O13" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P13" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="Q13" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="R13" s="3"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.15">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>2.4705869247685183E-2</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G14" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" t="s">
         <v>37</v>
-      </c>
-      <c r="F14" t="s">
-        <v>63</v>
-      </c>
-      <c r="G14" t="s">
-        <v>31</v>
-      </c>
-      <c r="H14" t="s">
-        <v>49</v>
       </c>
       <c r="I14">
         <v>6</v>
@@ -2043,47 +1514,47 @@
         <v>4.3425288506944444E-2</v>
       </c>
       <c r="M14" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="N14" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="O14" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="P14" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q14" t="s">
         <v>40</v>
       </c>
-      <c r="Q14" t="s">
-        <v>54</v>
-      </c>
       <c r="R14" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>2.8567820729166669E-2</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" t="s">
         <v>28</v>
-      </c>
-      <c r="D15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H15" t="s">
-        <v>40</v>
       </c>
       <c r="I15">
         <v>6</v>
@@ -2092,455 +1563,425 @@
         <v>4.6624869594907407E-2</v>
       </c>
       <c r="M15" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="N15" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="O15" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="P15" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="Q15" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.15">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>2.9694549490740744E-2</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H16" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="I16">
         <v>6</v>
       </c>
       <c r="J16" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="L16" s="2">
         <v>5.4334596921296295E-2</v>
       </c>
       <c r="M16" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="N16" t="s">
+        <v>18</v>
+      </c>
+      <c r="O16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P16" t="s">
         <v>28</v>
       </c>
-      <c r="O16" t="s">
-        <v>29</v>
-      </c>
-      <c r="P16" t="s">
+      <c r="Q16" t="s">
         <v>40</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>54</v>
       </c>
       <c r="R16" s="3"/>
       <c r="S16" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="T16" s="3"/>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>4.0407245069444445E-2</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D17" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E17" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="F17" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G17" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="H17" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="I17">
         <v>5</v>
       </c>
+      <c r="J17" t="s">
+        <v>53</v>
+      </c>
       <c r="L17" s="2">
         <v>5.7693504467592596E-2</v>
       </c>
       <c r="M17" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="N17" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O17" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="P17" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="Q17" t="s">
+        <v>23</v>
+      </c>
+      <c r="R17" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="R17" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>4.6125193645833333E-2</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" t="s">
         <v>28</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" t="s">
-        <v>39</v>
-      </c>
-      <c r="G18" t="s">
-        <v>48</v>
-      </c>
-      <c r="H18" t="s">
-        <v>40</v>
       </c>
       <c r="I18">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>4.6997797349537039E-2</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F19" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" t="s">
         <v>39</v>
-      </c>
-      <c r="G19" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" t="s">
-        <v>53</v>
       </c>
       <c r="I19">
         <v>5</v>
       </c>
       <c r="J19" t="s">
-        <v>69</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.15">
+        <v>54</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M19" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>4.8755836944444443E-2</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s">
+        <v>27</v>
+      </c>
+      <c r="G20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" t="s">
         <v>37</v>
-      </c>
-      <c r="F20" t="s">
-        <v>39</v>
-      </c>
-      <c r="G20" t="s">
-        <v>31</v>
-      </c>
-      <c r="H20" t="s">
-        <v>49</v>
       </c>
       <c r="I20">
         <v>6</v>
       </c>
-      <c r="L20" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="M20" s="8">
-        <f>COUNTIFS(DetailMelees[Introduction pour],"N",DetailMelees[Issue],"G")</f>
+      <c r="L20" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M20" s="7">
         <v>9</v>
       </c>
-      <c r="N20" s="8">
-        <f>COUNTIFS(DetailMelees[Introduction pour],"N",DetailMelees[Issue],"P")</f>
+      <c r="N20" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>5.1981994560185193E-2</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H21" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="I21">
         <v>5</v>
       </c>
-      <c r="L21" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="M21" s="10">
-        <f>COUNTIFS(DetailMelees[Introduction pour],"E",DetailMelees[Issue],"P")</f>
+      <c r="L21" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="M21" s="9">
         <v>6</v>
       </c>
-      <c r="N21" s="10">
-        <f>COUNTIFS(DetailMelees[Introduction pour],"E",DetailMelees[Issue],"G")</f>
+      <c r="N21" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>5.5310557418981485E-2</v>
       </c>
       <c r="B22" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D22" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G22" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H22" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="I22">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>5.7266875451388886E-2</v>
       </c>
       <c r="B23" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C23" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>42</v>
+      </c>
+      <c r="F23" t="s">
+        <v>27</v>
       </c>
       <c r="H23" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="I23">
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>6.0771433668981488E-2</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" t="s">
+        <v>27</v>
+      </c>
+      <c r="G24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" t="s">
         <v>37</v>
-      </c>
-      <c r="F24" t="s">
-        <v>39</v>
-      </c>
-      <c r="G24" t="s">
-        <v>31</v>
-      </c>
-      <c r="H24" t="s">
-        <v>49</v>
       </c>
       <c r="I24">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A25" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A26" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B26" s="14">
-        <f>COUNTIFS(DetailTouches[Lance pour],"N",DetailTouches[Issue],"G")</f>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A26" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A27" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="13">
         <v>3</v>
       </c>
-      <c r="C26" s="14">
-        <f>COUNTIFS(DetailTouches[Lance pour],"N",DetailTouches[Issue],"P")</f>
+      <c r="C27" s="13">
         <v>4</v>
       </c>
-      <c r="D26" s="14">
-        <f>COUNTIFS(DetailTouches[Lance pour],"N",DetailTouches[Issue],"ND")</f>
+      <c r="D27" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A27" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B27" s="10">
-        <f>COUNTIFS(DetailTouches[Lance pour],"E",DetailTouches[Issue],"P")</f>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A28" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="9">
         <v>7</v>
       </c>
-      <c r="C27" s="10">
-        <f>COUNTIFS(DetailTouches[Lance pour],"E",DetailTouches[Issue],"G")</f>
+      <c r="C28" s="9">
         <v>6</v>
       </c>
-      <c r="D27" s="10">
-        <f>COUNTIFS(DetailTouches[Lance pour],"E",DetailTouches[Issue],"ND")</f>
+      <c r="D28" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D3:D24">
-    <cfRule type="expression" dxfId="14" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="1" stopIfTrue="1">
       <formula>($C3&amp;$D3)="NP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="2" stopIfTrue="1">
       <formula>($C3&amp;$D3)="EG"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G24">
-    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="3" stopIfTrue="1">
       <formula>$G3="F"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="4" stopIfTrue="1">
       <formula>$G3="C"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:J24">
-    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="5" stopIfTrue="1">
       <formula>$C3="N"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="6" stopIfTrue="1">
       <formula>$C3&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O3:O17">
-    <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="7" stopIfTrue="1">
       <formula>($N3&amp;$O3)="NP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="8" stopIfTrue="1">
       <formula>($N3&amp;$O3)="EG"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L3:U17">
-    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="9" stopIfTrue="1">
       <formula>$N3="N"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="10" stopIfTrue="1">
       <formula>$N3&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I24" xr:uid="{3718F369-A628-514A-9BB0-869BD5FEF61D}">
-      <formula1>$AC$2:$AC$7</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G24" xr:uid="{2FC08E72-4ABE-2847-813E-C70CEC18990A}">
-      <formula1>$AA$2:$AA$3</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F24" xr:uid="{835BFA78-F23E-3842-8B29-DF13EF2DCBFC}">
-      <formula1>$Z$2:$Z$6</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D24" xr:uid="{67CA3FAE-529A-324E-A0BA-18E63C5787EE}">
-      <formula1>$X$2:$X$4</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q3:Q17" xr:uid="{09FB35A7-A0C8-A848-9382-5C1037E0E931}">
-      <formula1>$AD$2:$AD$4</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O3:O17" xr:uid="{8CDEC351-3A92-8A4A-A65F-10A97831BE25}">
-      <formula1>$Y$2:$Y$3</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:P17 H3:H24" xr:uid="{CAA819C7-5B3C-A543-896F-1C5B4EB3CD86}">
-      <formula1>$AB$2:$AB$12</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N17 C3:C24" xr:uid="{3B23A6AC-5D94-9F43-8FFA-F3807C07E58B}">
-      <formula1>$W$2:$W$3</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
     <tablePart r:id="rId1"/>

</xml_diff>